<commit_message>
Strip status-column hints from schedule_read timeline
The status column previously contained explicit annotations naming
each scheduling issue (e.g. "planned (overlaps M-Mill-B with P-003
Drilling)"). This made the task reading comprehension rather than
analytical reasoning.

Status values are now neutral labels only: done, planned, delayed,
blocked. The LLM must derive all four issues from the temporal and
resource data — date overlaps, sequence violations, and uncascaded
delays — without hints.

Ground truth keywords unchanged; all issues remain discoverable
from the raw date/machine/supplier columns.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/schedule_read/timeline.xlsx
+++ b/data/schedule_read/timeline.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Gantt" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Project Gantt" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>delayed (supplier 7 days late)</t>
+          <t>delayed</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>blocked (waiting for upstream)</t>
+          <t>blocked</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1113,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>planned (overlaps M-Mill-B with P-003 Drilling)</t>
+          <t>planned</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>planned (starts before Cutting predecessor finishes)</t>
+          <t>planned</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>delayed (8 days late, cascades downstream)</t>
+          <t>delayed</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>planned (date NOT rebaselined despite upstream delay)</t>
+          <t>planned</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>planned (date NOT rebaselined despite upstream delay)</t>
+          <t>planned</t>
         </is>
       </c>
     </row>

</xml_diff>